<commit_message>
refactor: improve accessibility and table layout handling
- Replace label with span and add ARIA attributes for better accessibility
- Simplify table layout logic in data-op.js and add ellipsis for overflow
- Add input IDs for Choices.js search inputs to improve form accessibility
- Adjust panel heights and overflow settings for better UI consistency
- Move records display logic to after panel animation completes
</commit_message>
<xml_diff>
--- a/tests/fused.xlsx
+++ b/tests/fused.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\acheng_work\test\git\git\my\perf_manager\test_case\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\acheng_work\test\git\git\my\perf_manager\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E89D03-83D6-4F4F-9024-0600E0470468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF5E49DA-2A93-45BE-A023-6671408547CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Total Ops(Mops)</t>
   </si>
@@ -92,6 +92,38 @@
   </si>
   <si>
     <t>NPU</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>qwertyuiop asdfghjkl zxcvbnm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>asd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ggg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>wwwww</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6.8.9.123</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>zsfgqweg asd2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>mko2sfgase</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gytr125</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -433,7 +465,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA7D009-FDBD-4201-92E5-251A772B1A94}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.08203125" customWidth="1"/>
@@ -444,7 +476,7 @@
     <col min="6" max="6" width="14.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -466,8 +498,29 @@
       <c r="G1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1">
+        <v>767334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0.46</v>
       </c>
@@ -488,6 +541,27 @@
       </c>
       <c r="G2" s="2">
         <v>8.1600000000000006E-2</v>
+      </c>
+      <c r="H2">
+        <v>33</v>
+      </c>
+      <c r="I2">
+        <v>1.4</v>
+      </c>
+      <c r="J2">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2">
+        <v>890</v>
+      </c>
+      <c r="N2">
+        <v>767334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>